<commit_message>
feat: adding link to import error message when a concept is not found by label
</commit_message>
<xml_diff>
--- a/src/main/resources/datasets/Import_Chartres_Projet.xlsx
+++ b/src/main/resources/datasets/Import_Chartres_Projet.xlsx
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C2" t="inlineStr" s="34">
         <is>
-          <t>US</t>
+          <t>Type inexistant TEST</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="36">
@@ -3815,8 +3815,10 @@
         </is>
       </c>
       <c r="E5" s="37"/>
-      <c r="F5" t="s" s="39">
-        <v>81</v>
+      <c r="F5" t="inlineStr" s="39">
+        <is>
+          <t>Interprétation inexistante TEST</t>
+        </is>
       </c>
       <c r="G5" t="s" s="6">
         <v>72</v>

</xml_diff>